<commit_message>
Verify document-accessibility kit and link it from its niche
Re-ran the full sample demo on a copy (crawl, triage, basic fixes,
tagged PDF export, snapshot report and remediation log).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/pdf-binder/samples/om-handover/output/SAMPLE_OM-Manual_Harborview-Clinic_Div-23-HVAC-index.xlsx
+++ b/kits/pdf-binder/samples/om-handover/output/SAMPLE_OM-Manual_Harborview-Clinic_Div-23-HVAC-index.xlsx
@@ -140,7 +140,7 @@
     <t>rtu-480-datasheet.pdf</t>
   </si>
   <si>
-    <t>65b7d0108724314c3d0a8d7226a1cec5afd7f9b49451016a7a742e3e1322e996</t>
+    <t>28c8aa0be17b341ea8b8a6c0f0e7e0bc4203c9f0907144c77f5bb39b2098604d</t>
   </si>
   <si>
     <t>2.2</t>
@@ -155,7 +155,7 @@
     <t>rtu-480-iom-manual.pdf</t>
   </si>
   <si>
-    <t>da2e6bfae149246fd9dc2b12aeb32043ea14d77d9d8f712dc7393fb62f2f0abf</t>
+    <t>e12ee333cc15d42c2fa6b2b282535e4d856653710f3cf8c55d27384b5277ae14</t>
   </si>
   <si>
     <t>2.3</t>
@@ -170,7 +170,7 @@
     <t>rtu-1-warranty.pdf</t>
   </si>
   <si>
-    <t>eb0215a4b34ce1512a290160dd76979487179393385914e34e046f3861321894</t>
+    <t>b4e83bfad50ea6e26b984db9d2d86d8ace334cbce14906c9733a9ad08828628c</t>
   </si>
   <si>
     <t>3</t>
@@ -194,7 +194,7 @@
     <t>ef-12-datasheet-A4.pdf</t>
   </si>
   <si>
-    <t>a2421e907135bed6e90eda6ae337910ea93d6844d84f912142b1476c9ee4241d</t>
+    <t>b5766f09d23c3e8156959c451fa5c252951ba4b57e76a721eaa587bc5df35ebb</t>
   </si>
   <si>
     <t>3.2</t>
@@ -206,7 +206,7 @@
     <t>ef-12-manual.pdf</t>
   </si>
   <si>
-    <t>e18c6094701f493832de3309b3f64d87dc831cfdb4e3a4735b70f7ce70e54a52</t>
+    <t>f313d041bc849d841f0b0492867616e009e99a26a1107267eddbdd700d636008</t>
   </si>
   <si>
     <t>3.3</t>
@@ -218,7 +218,7 @@
     <t>ef-warranty.pdf</t>
   </si>
   <si>
-    <t>f0bd96248ac50c5191977e6befc4c5b84c75dc96ac257cd20ab48ae5db8a1f91</t>
+    <t>b1e32524e0920f7d5a1250c7262fa79bb0ce6231ab8555414cbf13ed50096812</t>
   </si>
   <si>
     <t>4</t>
@@ -239,7 +239,7 @@
     <t>vav-s-datasheet.pdf</t>
   </si>
   <si>
-    <t>59c8de42fee564f97eeff37083579c3e3c2375d7f750c7ff27e15da11ca9f22e</t>
+    <t>850763cd0d3b2827dce1541372918235417527083c813805c241e06aa30f2f80</t>
   </si>
   <si>
     <t>4.2</t>
@@ -248,7 +248,7 @@
     <t>vav-s-manual.pdf</t>
   </si>
   <si>
-    <t>577c8e3552e1ab2a0c4be46ce6327c5cb8aad2c29b5378b4699d1d9ef6c4a152</t>
+    <t>b1e36b10621c874e3cd971f1b235038300f00e88258f229e306c5f7a092658fe</t>
   </si>
   <si>
     <t>5</t>
@@ -269,7 +269,7 @@
     <t>t200-thermostat-datasheet.pdf</t>
   </si>
   <si>
-    <t>626f802bd4d541fcd4fede86d9217fba14fe78bc316f7b63ef5afb874e807911</t>
+    <t>7b4e3da98e45bac4a41a8d1262996387eacd6698e164980a642c0d4c31150e1e</t>
   </si>
   <si>
     <t>5.2</t>
@@ -284,7 +284,7 @@
     <t>sequence-of-operations.pdf</t>
   </si>
   <si>
-    <t>7cdd2fe1e47afd60f3798845d58ea9465583c95da6792561376d14c7c6e12b6f</t>
+    <t>155e5ad57c31879e0c1e980b18734215266fa2713b34fc5c1b8850987c513ea4</t>
   </si>
   <si>
     <t>6</t>
@@ -383,7 +383,7 @@
     <t>m-101-record-drawing.pdf</t>
   </si>
   <si>
-    <t>a12a1be2cb135b2b88b9b43442ece044b63a6664aace4269ef2760e3e5ced65f</t>
+    <t>52849f6767b705adfaa76f349240aaa1c5aae98d4f5341542384893f18306f1e</t>
   </si>
   <si>
     <t>Binder summary</t>
@@ -404,7 +404,7 @@
     <t>Built on</t>
   </si>
   <si>
-    <t>2026-10-07 10:35</t>
+    <t>2026-10-07 10:36</t>
   </si>
   <si>
     <t>Total pages</t>

</xml_diff>

<commit_message>
Verify PDF binder kit, link it, and fix LibreOffice Writer note
The PDF binder tests pass and the three sample binders rebuild with
every verify check passing. A fresh cloud session has only part of
LibreOffice, so the board-minutes kit now says to install Writer for
PDFs and its setup script checks for it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DspfyLwNfeJ4CHdyACeRHQ
</commit_message>
<xml_diff>
--- a/kits/pdf-binder/samples/om-handover/output/SAMPLE_OM-Manual_Harborview-Clinic_Div-23-HVAC-index.xlsx
+++ b/kits/pdf-binder/samples/om-handover/output/SAMPLE_OM-Manual_Harborview-Clinic_Div-23-HVAC-index.xlsx
@@ -140,7 +140,7 @@
     <t>rtu-480-datasheet.pdf</t>
   </si>
   <si>
-    <t>28c8aa0be17b341ea8b8a6c0f0e7e0bc4203c9f0907144c77f5bb39b2098604d</t>
+    <t>7601b79382acdadbcbf5a22abfe2c4613ffd9dd7e3b9b7b6538818222dc7a0eb</t>
   </si>
   <si>
     <t>2.2</t>
@@ -155,7 +155,7 @@
     <t>rtu-480-iom-manual.pdf</t>
   </si>
   <si>
-    <t>e12ee333cc15d42c2fa6b2b282535e4d856653710f3cf8c55d27384b5277ae14</t>
+    <t>c94b979d907ecf41740802b456bc162cd9dafac0e900b7a3dceda5ff2585b31f</t>
   </si>
   <si>
     <t>2.3</t>
@@ -170,7 +170,7 @@
     <t>rtu-1-warranty.pdf</t>
   </si>
   <si>
-    <t>b4e83bfad50ea6e26b984db9d2d86d8ace334cbce14906c9733a9ad08828628c</t>
+    <t>161c90133519b038b6df5434f0612f3acd16d05dea92355c3a18aeab8d1899f6</t>
   </si>
   <si>
     <t>3</t>
@@ -194,7 +194,7 @@
     <t>ef-12-datasheet-A4.pdf</t>
   </si>
   <si>
-    <t>b5766f09d23c3e8156959c451fa5c252951ba4b57e76a721eaa587bc5df35ebb</t>
+    <t>ba70aff223666f818e1398425f269c8a4a82cbb633e1cf6c0e225f464ee4e71b</t>
   </si>
   <si>
     <t>3.2</t>
@@ -206,7 +206,7 @@
     <t>ef-12-manual.pdf</t>
   </si>
   <si>
-    <t>f313d041bc849d841f0b0492867616e009e99a26a1107267eddbdd700d636008</t>
+    <t>21c81991ef18231a1fdb7d304e7d1ce3ed480ebefa518ff3606242f8bb443e0b</t>
   </si>
   <si>
     <t>3.3</t>
@@ -218,7 +218,7 @@
     <t>ef-warranty.pdf</t>
   </si>
   <si>
-    <t>b1e32524e0920f7d5a1250c7262fa79bb0ce6231ab8555414cbf13ed50096812</t>
+    <t>4ea7a27e54968e33dfb219726a3f63034b7daabdea828c3fe8d858aee6ddd7f5</t>
   </si>
   <si>
     <t>4</t>
@@ -239,7 +239,7 @@
     <t>vav-s-datasheet.pdf</t>
   </si>
   <si>
-    <t>850763cd0d3b2827dce1541372918235417527083c813805c241e06aa30f2f80</t>
+    <t>eda99d68e77c66ed0cc5864fd08d9609aa9bc5cde01a4a3736df53f3f4d6c508</t>
   </si>
   <si>
     <t>4.2</t>
@@ -248,7 +248,7 @@
     <t>vav-s-manual.pdf</t>
   </si>
   <si>
-    <t>b1e36b10621c874e3cd971f1b235038300f00e88258f229e306c5f7a092658fe</t>
+    <t>8bef2637b571826777d79f22f9f62c48a0b9e36ad61cfcbdcfbbf1cd89c63800</t>
   </si>
   <si>
     <t>5</t>
@@ -269,7 +269,7 @@
     <t>t200-thermostat-datasheet.pdf</t>
   </si>
   <si>
-    <t>7b4e3da98e45bac4a41a8d1262996387eacd6698e164980a642c0d4c31150e1e</t>
+    <t>85a1803b2b8507a8b32998da6a02c0df1878973cecc44c3e480023c794717149</t>
   </si>
   <si>
     <t>5.2</t>
@@ -284,7 +284,7 @@
     <t>sequence-of-operations.pdf</t>
   </si>
   <si>
-    <t>155e5ad57c31879e0c1e980b18734215266fa2713b34fc5c1b8850987c513ea4</t>
+    <t>ce61e23314973f8faa3fdd717d556cce36f5c7586533a4363daca57155a259cf</t>
   </si>
   <si>
     <t>6</t>
@@ -383,7 +383,7 @@
     <t>m-101-record-drawing.pdf</t>
   </si>
   <si>
-    <t>52849f6767b705adfaa76f349240aaa1c5aae98d4f5341542384893f18306f1e</t>
+    <t>6cd50d99589cec17ae4223214c570a3fe97d36233bb5a2c88040886d681ce979</t>
   </si>
   <si>
     <t>Binder summary</t>
@@ -404,7 +404,7 @@
     <t>Built on</t>
   </si>
   <si>
-    <t>2026-10-07 10:36</t>
+    <t>2026-10-07 10:49</t>
   </si>
   <si>
     <t>Total pages</t>

</xml_diff>